<commit_message>
interfaz con arrastre de archivos, y aplicacion de incrementos a varias grillas
</commit_message>
<xml_diff>
--- a/PRUEBA.xlsx
+++ b/PRUEBA.xlsx
@@ -15,11 +15,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;\ #,##0.00;[Red]\-&quot;$&quot;\ #,##0.00"/>
     <numFmt numFmtId="166" formatCode="DD/MM/YYYY"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -511,7 +510,7 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="n">
-        <v>20106</v>
+        <v>31164.3</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -571,7 +570,7 @@
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="n">
-        <v>20202</v>
+        <v>31313.1</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -631,7 +630,7 @@
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="n">
-        <v>20301</v>
+        <v>31466.55</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -691,7 +690,7 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="n">
-        <v>20403</v>
+        <v>31624.65</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -751,7 +750,7 @@
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="n">
-        <v>20502</v>
+        <v>31778.1</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -811,7 +810,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>20602</v>
+        <v>31933.1</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
@@ -819,39 +818,39 @@
         </is>
       </c>
       <c r="C7" s="8" t="n">
-        <v>213831.22</v>
+        <v>331438.391</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>245905.903</v>
+        <v>381154.14965</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>282791.78845</v>
+        <v>438327.2720975</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>353489.7355625</v>
+        <v>547909.0901218751</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>459536.65623125</v>
+        <v>712281.8171584375</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>597397.653100625</v>
+        <v>925966.3623059688</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>776616.9490308126</v>
+        <v>1203756.27099776</v>
       </c>
       <c r="J7" s="8" t="n">
-        <v>854278.6439338939</v>
+        <v>1324131.898097536</v>
       </c>
       <c r="K7" s="8" t="n">
-        <v>1110562.237114062</v>
+        <v>1721371.467526796</v>
       </c>
       <c r="L7" s="8" t="n">
-        <v>1443730.908248281</v>
+        <v>2237782.907784836</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="n">
-        <v>20801</v>
+        <v>32241.55</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
@@ -911,7 +910,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>25006</v>
+        <v>38759.3</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -919,39 +918,39 @@
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>376060.25</v>
+        <v>582893.3875000001</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>432469.2875</v>
+        <v>670327.395625</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>497339.6806249999</v>
+        <v>770876.5049687499</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>621674.6007812499</v>
+        <v>963595.6312109374</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>808176.9810156249</v>
+        <v>1252674.320574219</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>1050630.075320313</v>
+        <v>1628476.616746485</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>1365819.097916407</v>
+        <v>2117019.601770431</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>1502401.007708048</v>
+        <v>2328721.561947474</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>1953121.310020462</v>
+        <v>3027338.030531716</v>
       </c>
       <c r="L9" s="8" t="n">
-        <v>2539057.703026601</v>
+        <v>3935539.439691232</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>25601</v>
+        <v>39681.55</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -959,39 +958,39 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>213831.22</v>
+        <v>331438.391</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>245905.903</v>
+        <v>381154.14965</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>282791.78845</v>
+        <v>438327.2720975</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>353489.7355625</v>
+        <v>547909.0901218751</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>459536.65623125</v>
+        <v>712281.8171584375</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>597397.653100625</v>
+        <v>925966.3623059688</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>776616.9490308126</v>
+        <v>1203756.27099776</v>
       </c>
       <c r="J10" s="8" t="n">
-        <v>854278.6439338939</v>
+        <v>1324131.898097536</v>
       </c>
       <c r="K10" s="8" t="n">
-        <v>1110562.237114062</v>
+        <v>1721371.467526796</v>
       </c>
       <c r="L10" s="8" t="n">
-        <v>1443730.908248281</v>
+        <v>2237782.907784836</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>25608</v>
+        <v>39692.4</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -999,39 +998,39 @@
         </is>
       </c>
       <c r="C11" s="8" t="n">
-        <v>691567.2</v>
+        <v>1071929.16</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>795302.2799999999</v>
+        <v>1232718.534</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>914597.6219999999</v>
+        <v>1417626.3141</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>1143247.0275</v>
+        <v>1772032.892625</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>1486221.13575</v>
+        <v>2303642.7604125</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>1932087.476475</v>
+        <v>2994735.58853625</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>2511713.7194175</v>
+        <v>3893156.265097125</v>
       </c>
       <c r="J11" s="8" t="n">
-        <v>2762885.09135925</v>
+        <v>4282471.891606838</v>
       </c>
       <c r="K11" s="8" t="n">
-        <v>3591750.618767025</v>
+        <v>5567213.459088889</v>
       </c>
       <c r="L11" s="8" t="n">
-        <v>4669275.804397132</v>
+        <v>7237377.496815555</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2" t="n">
-        <v>25805</v>
+        <v>39997.75</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -1091,7 +1090,7 @@
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="2" t="n">
-        <v>25808</v>
+        <v>40002.4</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
@@ -1151,7 +1150,7 @@
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="2" t="n">
-        <v>28002</v>
+        <v>43403.1</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -1211,7 +1210,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>28003</v>
+        <v>43404.65</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -1219,39 +1218,39 @@
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>1374307.23</v>
+        <v>2130176.2065</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>1580453.3145</v>
+        <v>2449702.637475</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>1817521.311675</v>
+        <v>2817158.03309625</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>2271901.63959375</v>
+        <v>3521447.541370312</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>2953472.131471875</v>
+        <v>4577881.803781407</v>
       </c>
       <c r="H15" s="8" t="n">
-        <v>3839513.770913438</v>
+        <v>5951246.344915829</v>
       </c>
       <c r="I15" s="8" t="n">
-        <v>4991367.902187469</v>
+        <v>7736620.248390578</v>
       </c>
       <c r="J15" s="8" t="n">
-        <v>5490504.692406217</v>
+        <v>8510282.273229636</v>
       </c>
       <c r="K15" s="8" t="n">
-        <v>7137656.100128082</v>
+        <v>11063366.95519853</v>
       </c>
       <c r="L15" s="8" t="n">
-        <v>9278952.930166507</v>
+        <v>14382377.04175809</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="2" t="n">
-        <v>28007</v>
+        <v>43410.85</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
@@ -1311,7 +1310,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>28016</v>
+        <v>43424.8</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
@@ -1319,39 +1318,39 @@
         </is>
       </c>
       <c r="C17" s="8" t="n">
-        <v>2351916.02</v>
+        <v>3645469.831</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>2704703.423</v>
+        <v>4192290.30565</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>3110408.93645</v>
+        <v>4821133.8514975</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>3888011.1705625</v>
+        <v>6026417.314371875</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>5054414.52173125</v>
+        <v>7834342.508683437</v>
       </c>
       <c r="H17" s="8" t="n">
-        <v>6570738.878250625</v>
+        <v>10184645.26128847</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>8541960.541725812</v>
+        <v>13240038.83967501</v>
       </c>
       <c r="J17" s="8" t="n">
-        <v>9396156.595898395</v>
+        <v>14564042.72364251</v>
       </c>
       <c r="K17" s="8" t="n">
-        <v>12215003.57466791</v>
+        <v>18933255.54073526</v>
       </c>
       <c r="L17" s="8" t="n">
-        <v>15879504.64706828</v>
+        <v>24613232.20295583</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2" t="n">
-        <v>28025</v>
+        <v>43438.75</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
@@ -1411,7 +1410,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>28029</v>
+        <v>43444.95</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
@@ -1419,39 +1418,39 @@
         </is>
       </c>
       <c r="C19" s="8" t="n">
-        <v>1177977.62</v>
+        <v>1825865.311</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>1354674.263</v>
+        <v>2099745.10765</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>1557875.40245</v>
+        <v>2414706.8737975</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>1947344.2530625</v>
+        <v>3018383.592246875</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>2531547.52898125</v>
+        <v>3923898.669920937</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>3291011.787675625</v>
+        <v>5101068.270897219</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>4278315.323978313</v>
+        <v>6631388.752166386</v>
       </c>
       <c r="J19" s="8" t="n">
-        <v>4706146.856376145</v>
+        <v>7294527.627383025</v>
       </c>
       <c r="K19" s="8" t="n">
-        <v>6117990.913288989</v>
+        <v>9482885.915597934</v>
       </c>
       <c r="L19" s="8" t="n">
-        <v>7953388.187275686</v>
+        <v>12327751.69027731</v>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="2" t="n">
-        <v>28049</v>
+        <v>43475.95</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
@@ -1511,7 +1510,7 @@
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="2" t="n">
-        <v>28056</v>
+        <v>43486.8</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
@@ -1571,7 +1570,7 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>28056</v>
+        <v>43486.8</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
@@ -1579,39 +1578,39 @@
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>292418.77</v>
+        <v>453249.0935</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>336281.5855</v>
+        <v>521236.457525</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>386723.8233249999</v>
+        <v>599421.9261537498</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>483404.7791562498</v>
+        <v>749277.4076921871</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>628426.2129031247</v>
+        <v>974060.6299998434</v>
       </c>
       <c r="H22" s="8" t="n">
-        <v>816954.0767740622</v>
+        <v>1266278.818999796</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>1062040.299806281</v>
+        <v>1646162.464699736</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>1168244.329786909</v>
+        <v>1810778.711169709</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>1518717.628722982</v>
+        <v>2354012.324520622</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>1974332.917339877</v>
+        <v>3060216.02187681</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>28057</v>
+        <v>43488.35</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
@@ -1619,39 +1618,39 @@
         </is>
       </c>
       <c r="C23" s="8" t="n">
-        <v>255866.42</v>
+        <v>396592.9510000001</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>294246.383</v>
+        <v>456081.89365</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>338383.34045</v>
+        <v>524494.1776975001</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>422979.1755625</v>
+        <v>655617.722121875</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>549872.92823125</v>
+        <v>852303.0387584376</v>
       </c>
       <c r="H23" s="8" t="n">
-        <v>714834.8067006251</v>
+        <v>1107993.950385969</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>929285.2487108127</v>
+        <v>1440392.13550176</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>1022213.773581894</v>
+        <v>1584431.349051936</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>1328877.905656462</v>
+        <v>2059760.753767516</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>1727541.277353401</v>
+        <v>2677688.979897771</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="2" t="n">
-        <v>28090</v>
+        <v>43539.5</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
@@ -1711,7 +1710,7 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>75722</v>
+        <v>117369.1</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
@@ -1719,39 +1718,39 @@
         </is>
       </c>
       <c r="C25" s="8" t="n">
-        <v>2838313.12</v>
+        <v>4399385.336</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>3264060.088</v>
+        <v>5059293.1364</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>3753669.1012</v>
+        <v>5818187.10686</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>4692086.3765</v>
+        <v>7272733.883575001</v>
       </c>
       <c r="G25" s="8" t="n">
-        <v>6099712.289450001</v>
+        <v>9454554.048647502</v>
       </c>
       <c r="H25" s="8" t="n">
-        <v>7929625.976285001</v>
+        <v>12290920.26324175</v>
       </c>
       <c r="I25" s="8" t="n">
-        <v>10308513.7691705</v>
+        <v>15978196.34221428</v>
       </c>
       <c r="J25" s="8" t="n">
-        <v>11339365.14608755</v>
+        <v>17576015.9764357</v>
       </c>
       <c r="K25" s="8" t="n">
-        <v>14741174.68991381</v>
+        <v>22848820.76936641</v>
       </c>
       <c r="L25" s="8" t="n">
-        <v>19163527.09688795</v>
+        <v>29703467.00017632</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>180109</v>
+        <v>279168.95</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
@@ -1759,39 +1758,39 @@
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>42217.47</v>
+        <v>65437.0785</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>48550.0905</v>
+        <v>75252.640275</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>55832.604075</v>
+        <v>86540.53631625</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>69790.75509375001</v>
+        <v>108175.6703953125</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>90727.98162187501</v>
+        <v>140628.3715139063</v>
       </c>
       <c r="H26" s="8" t="n">
-        <v>117946.3761084375</v>
+        <v>182816.8829680781</v>
       </c>
       <c r="I26" s="8" t="n">
-        <v>153330.2889409687</v>
+        <v>237661.9478585015</v>
       </c>
       <c r="J26" s="8" t="n">
-        <v>168663.3178350656</v>
+        <v>261428.1426443517</v>
       </c>
       <c r="K26" s="8" t="n">
-        <v>219262.3131855853</v>
+        <v>339856.5854376573</v>
       </c>
       <c r="L26" s="8" t="n">
-        <v>285041.0071412609</v>
+        <v>441813.5610689544</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>300111</v>
+        <v>465172.05</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
@@ -1799,39 +1798,39 @@
         </is>
       </c>
       <c r="C27" s="8" t="n">
-        <v>42217.47</v>
+        <v>65437.0785</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>48550.0905</v>
+        <v>75252.640275</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>55832.604075</v>
+        <v>86540.53631625</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>69790.75509375001</v>
+        <v>108175.6703953125</v>
       </c>
       <c r="G27" s="8" t="n">
-        <v>90727.98162187501</v>
+        <v>140628.3715139063</v>
       </c>
       <c r="H27" s="8" t="n">
-        <v>117946.3761084375</v>
+        <v>182816.8829680781</v>
       </c>
       <c r="I27" s="8" t="n">
-        <v>153330.2889409687</v>
+        <v>237661.9478585015</v>
       </c>
       <c r="J27" s="8" t="n">
-        <v>168663.3178350656</v>
+        <v>261428.1426443517</v>
       </c>
       <c r="K27" s="8" t="n">
-        <v>219262.3131855853</v>
+        <v>339856.5854376573</v>
       </c>
       <c r="L27" s="8" t="n">
-        <v>285041.0071412609</v>
+        <v>441813.5610689544</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>300112</v>
+        <v>465173.6</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
@@ -1839,39 +1838,39 @@
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>22845.22</v>
+        <v>35410.091</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>26272.003</v>
+        <v>40721.60465</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>30212.80345</v>
+        <v>46829.8453475</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>37766.0043125</v>
+        <v>58537.30668437501</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>49095.80560625</v>
+        <v>76098.49868968751</v>
       </c>
       <c r="H28" s="8" t="n">
-        <v>63824.54728812501</v>
+        <v>98928.04829659377</v>
       </c>
       <c r="I28" s="8" t="n">
-        <v>82971.91147456251</v>
+        <v>128606.4627855719</v>
       </c>
       <c r="J28" s="8" t="n">
-        <v>91269.10262201878</v>
+        <v>141467.1090641291</v>
       </c>
       <c r="K28" s="8" t="n">
-        <v>118649.8334086244</v>
+        <v>183907.2417833678</v>
       </c>
       <c r="L28" s="8" t="n">
-        <v>154244.7834312117</v>
+        <v>239079.4143183781</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>300113</v>
+        <v>465175.15</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
@@ -1879,39 +1878,39 @@
         </is>
       </c>
       <c r="C29" s="8" t="n">
-        <v>42217.47</v>
+        <v>65437.0785</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>48550.0905</v>
+        <v>75252.640275</v>
       </c>
       <c r="E29" s="8" t="n">
-        <v>55832.604075</v>
+        <v>86540.53631625</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>69790.75509375001</v>
+        <v>108175.6703953125</v>
       </c>
       <c r="G29" s="8" t="n">
-        <v>90727.98162187501</v>
+        <v>140628.3715139063</v>
       </c>
       <c r="H29" s="8" t="n">
-        <v>117946.3761084375</v>
+        <v>182816.8829680781</v>
       </c>
       <c r="I29" s="8" t="n">
-        <v>153330.2889409687</v>
+        <v>237661.9478585015</v>
       </c>
       <c r="J29" s="8" t="n">
-        <v>168663.3178350656</v>
+        <v>261428.1426443517</v>
       </c>
       <c r="K29" s="8" t="n">
-        <v>219262.3131855853</v>
+        <v>339856.5854376573</v>
       </c>
       <c r="L29" s="8" t="n">
-        <v>285041.0071412609</v>
+        <v>441813.5610689544</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>305001</v>
+        <v>472751.55</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
@@ -1919,39 +1918,39 @@
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>29227.48</v>
+        <v>45302.594</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>33611.602</v>
+        <v>52097.9831</v>
       </c>
       <c r="E30" s="8" t="n">
-        <v>38653.3423</v>
+        <v>59912.680565</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>48316.67787499999</v>
+        <v>74890.85070624998</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>62811.68123749999</v>
+        <v>97358.10591812499</v>
       </c>
       <c r="H30" s="8" t="n">
-        <v>81655.18560874999</v>
+        <v>126565.5376935625</v>
       </c>
       <c r="I30" s="8" t="n">
-        <v>106151.741291375</v>
+        <v>164535.1990016313</v>
       </c>
       <c r="J30" s="8" t="n">
-        <v>116766.9154205125</v>
+        <v>180988.7189017944</v>
       </c>
       <c r="K30" s="8" t="n">
-        <v>151796.9900466662</v>
+        <v>235285.3345723326</v>
       </c>
       <c r="L30" s="8" t="n">
-        <v>197336.0870606661</v>
+        <v>305870.9349440325</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>305004</v>
+        <v>472756.2</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
@@ -1959,39 +1958,39 @@
         </is>
       </c>
       <c r="C31" s="8" t="n">
-        <v>29227.48</v>
+        <v>45302.594</v>
       </c>
       <c r="D31" s="8" t="n">
-        <v>33611.602</v>
+        <v>52097.9831</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>38653.3423</v>
+        <v>59912.680565</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>48316.67787499999</v>
+        <v>74890.85070624998</v>
       </c>
       <c r="G31" s="8" t="n">
-        <v>62811.68123749999</v>
+        <v>97358.10591812499</v>
       </c>
       <c r="H31" s="8" t="n">
-        <v>81655.18560874999</v>
+        <v>126565.5376935625</v>
       </c>
       <c r="I31" s="8" t="n">
-        <v>106151.741291375</v>
+        <v>164535.1990016313</v>
       </c>
       <c r="J31" s="8" t="n">
-        <v>116766.9154205125</v>
+        <v>180988.7189017944</v>
       </c>
       <c r="K31" s="8" t="n">
-        <v>151796.9900466662</v>
+        <v>235285.3345723326</v>
       </c>
       <c r="L31" s="8" t="n">
-        <v>197336.0870606661</v>
+        <v>305870.9349440325</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>305010</v>
+        <v>472765.5</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
@@ -1999,39 +1998,39 @@
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>29227.48</v>
+        <v>45302.594</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>33611.602</v>
+        <v>52097.9831</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>38653.3423</v>
+        <v>59912.680565</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>48316.67787499999</v>
+        <v>74890.85070624998</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>62811.68123749999</v>
+        <v>97358.10591812499</v>
       </c>
       <c r="H32" s="8" t="n">
-        <v>81655.18560874999</v>
+        <v>126565.5376935625</v>
       </c>
       <c r="I32" s="8" t="n">
-        <v>106151.741291375</v>
+        <v>164535.1990016313</v>
       </c>
       <c r="J32" s="8" t="n">
-        <v>116766.9154205125</v>
+        <v>180988.7189017944</v>
       </c>
       <c r="K32" s="8" t="n">
-        <v>151796.9900466662</v>
+        <v>235285.3345723326</v>
       </c>
       <c r="L32" s="8" t="n">
-        <v>197336.0870606661</v>
+        <v>305870.9349440325</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>305015</v>
+        <v>472773.25</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
@@ -2039,39 +2038,39 @@
         </is>
       </c>
       <c r="C33" s="8" t="n">
-        <v>29227.48</v>
+        <v>45302.594</v>
       </c>
       <c r="D33" s="8" t="n">
-        <v>33611.602</v>
+        <v>52097.9831</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>38653.3423</v>
+        <v>59912.680565</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>48316.67787499999</v>
+        <v>74890.85070624998</v>
       </c>
       <c r="G33" s="8" t="n">
-        <v>62811.68123749999</v>
+        <v>97358.10591812499</v>
       </c>
       <c r="H33" s="8" t="n">
-        <v>81655.18560874999</v>
+        <v>126565.5376935625</v>
       </c>
       <c r="I33" s="8" t="n">
-        <v>106151.741291375</v>
+        <v>164535.1990016313</v>
       </c>
       <c r="J33" s="8" t="n">
-        <v>116766.9154205125</v>
+        <v>180988.7189017944</v>
       </c>
       <c r="K33" s="8" t="n">
-        <v>151796.9900466662</v>
+        <v>235285.3345723326</v>
       </c>
       <c r="L33" s="8" t="n">
-        <v>197336.0870606661</v>
+        <v>305870.9349440325</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>305027</v>
+        <v>472791.85</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
@@ -2079,39 +2078,39 @@
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>64949.96</v>
+        <v>100672.438</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>74692.454</v>
+        <v>115773.3037</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>85896.32209999999</v>
+        <v>133139.299255</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>107370.402625</v>
+        <v>166424.12406875</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>139581.5234125</v>
+        <v>216351.361289375</v>
       </c>
       <c r="H34" s="8" t="n">
-        <v>181455.98043625</v>
+        <v>281256.7696761875</v>
       </c>
       <c r="I34" s="8" t="n">
-        <v>235892.774567125</v>
+        <v>365633.8005790437</v>
       </c>
       <c r="J34" s="8" t="n">
-        <v>259482.0520238375</v>
+        <v>402197.1806369481</v>
       </c>
       <c r="K34" s="8" t="n">
-        <v>337326.6676309888</v>
+        <v>522856.3348280327</v>
       </c>
       <c r="L34" s="8" t="n">
-        <v>438524.6679202855</v>
+        <v>679713.2352764425</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>305029</v>
+        <v>472794.95</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
@@ -2119,39 +2118,39 @@
         </is>
       </c>
       <c r="C35" s="8" t="n">
-        <v>97424.94</v>
+        <v>151008.657</v>
       </c>
       <c r="D35" s="8" t="n">
-        <v>112038.681</v>
+        <v>173659.95555</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>128844.48315</v>
+        <v>199708.9488825</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>161055.6039375</v>
+        <v>249636.186103125</v>
       </c>
       <c r="G35" s="8" t="n">
-        <v>209372.28511875</v>
+        <v>324527.0419340625</v>
       </c>
       <c r="H35" s="8" t="n">
-        <v>272183.970654375</v>
+        <v>421885.1545142813</v>
       </c>
       <c r="I35" s="8" t="n">
-        <v>353839.1618506875</v>
+        <v>548450.7008685657</v>
       </c>
       <c r="J35" s="8" t="n">
-        <v>389223.0780357563</v>
+        <v>603295.7709554223</v>
       </c>
       <c r="K35" s="8" t="n">
-        <v>505990.0014464832</v>
+        <v>784284.502242049</v>
       </c>
       <c r="L35" s="8" t="n">
-        <v>657787.0018804282</v>
+        <v>1019569.852914664</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>305038</v>
+        <v>472808.9</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
@@ -2159,39 +2158,39 @@
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>42217.47</v>
+        <v>65437.0785</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>48550.0905</v>
+        <v>75252.640275</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>55832.604075</v>
+        <v>86540.53631625</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>69790.75509375001</v>
+        <v>108175.6703953125</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>90727.98162187501</v>
+        <v>140628.3715139063</v>
       </c>
       <c r="H36" s="8" t="n">
-        <v>117946.3761084375</v>
+        <v>182816.8829680781</v>
       </c>
       <c r="I36" s="8" t="n">
-        <v>153330.2889409687</v>
+        <v>237661.9478585015</v>
       </c>
       <c r="J36" s="8" t="n">
-        <v>168663.3178350656</v>
+        <v>261428.1426443517</v>
       </c>
       <c r="K36" s="8" t="n">
-        <v>219262.3131855853</v>
+        <v>339856.5854376573</v>
       </c>
       <c r="L36" s="8" t="n">
-        <v>285041.0071412609</v>
+        <v>441813.5610689544</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>305043</v>
+        <v>472816.65</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
@@ -2199,39 +2198,39 @@
         </is>
       </c>
       <c r="C37" s="8" t="n">
-        <v>71444.95</v>
+        <v>110739.6725</v>
       </c>
       <c r="D37" s="8" t="n">
-        <v>82161.69249999999</v>
+        <v>127350.623375</v>
       </c>
       <c r="E37" s="8" t="n">
-        <v>94485.94637499998</v>
+        <v>146453.21688125</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>118107.43296875</v>
+        <v>183066.5211015625</v>
       </c>
       <c r="G37" s="8" t="n">
-        <v>153539.662859375</v>
+        <v>237986.4774320313</v>
       </c>
       <c r="H37" s="8" t="n">
-        <v>199601.5617171875</v>
+        <v>309382.4206616406</v>
       </c>
       <c r="I37" s="8" t="n">
-        <v>259482.0302323437</v>
+        <v>402197.1468601328</v>
       </c>
       <c r="J37" s="8" t="n">
-        <v>285430.2332555781</v>
+        <v>442416.861546146</v>
       </c>
       <c r="K37" s="8" t="n">
-        <v>371059.3032322516</v>
+        <v>575141.92000999</v>
       </c>
       <c r="L37" s="8" t="n">
-        <v>482377.0942019271</v>
+        <v>747684.496012987</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>305043</v>
+        <v>472816.65</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
@@ -2239,39 +2238,39 @@
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>81187.45</v>
+        <v>125840.5475</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>93365.56749999999</v>
+        <v>144716.629625</v>
       </c>
       <c r="E38" s="8" t="n">
-        <v>107370.402625</v>
+        <v>166424.12406875</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>134213.00328125</v>
+        <v>208030.1550859375</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>174476.904265625</v>
+        <v>270439.2016117187</v>
       </c>
       <c r="H38" s="8" t="n">
-        <v>226819.9755453125</v>
+        <v>351570.9620952344</v>
       </c>
       <c r="I38" s="8" t="n">
-        <v>294865.9682089063</v>
+        <v>457042.2507238048</v>
       </c>
       <c r="J38" s="8" t="n">
-        <v>324352.565029797</v>
+        <v>502746.4757961854</v>
       </c>
       <c r="K38" s="8" t="n">
-        <v>421658.3345387361</v>
+        <v>653570.4185350409</v>
       </c>
       <c r="L38" s="8" t="n">
-        <v>548155.8349003569</v>
+        <v>849641.5440955533</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>305044</v>
+        <v>472818.2</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
@@ -2279,39 +2278,39 @@
         </is>
       </c>
       <c r="C39" s="8" t="n">
-        <v>40593.74</v>
+        <v>62920.297</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>46682.80099999999</v>
+        <v>72358.34154999998</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>53685.22114999999</v>
+        <v>83212.09278249998</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>67106.52643749998</v>
+        <v>104015.115978125</v>
       </c>
       <c r="G39" s="8" t="n">
-        <v>87238.48436874998</v>
+        <v>135219.6507715625</v>
       </c>
       <c r="H39" s="8" t="n">
-        <v>113410.029679375</v>
+        <v>175785.5460030313</v>
       </c>
       <c r="I39" s="8" t="n">
-        <v>147433.0385831875</v>
+        <v>228521.2098039406</v>
       </c>
       <c r="J39" s="8" t="n">
-        <v>162176.3424415063</v>
+        <v>251373.3307843348</v>
       </c>
       <c r="K39" s="8" t="n">
-        <v>210829.2451739582</v>
+        <v>326785.3300196352</v>
       </c>
       <c r="L39" s="8" t="n">
-        <v>274078.0187261457</v>
+        <v>424820.9290255258</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>305045</v>
+        <v>472819.75</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
@@ -2319,39 +2318,39 @@
         </is>
       </c>
       <c r="C40" s="8" t="n">
-        <v>61702.46</v>
+        <v>95638.81299999999</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>70957.829</v>
+        <v>109984.63495</v>
       </c>
       <c r="E40" s="8" t="n">
-        <v>81601.50334999998</v>
+        <v>126482.3301925</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>102001.8791875</v>
+        <v>158102.912740625</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>132602.44294375</v>
+        <v>205533.7865628125</v>
       </c>
       <c r="H40" s="8" t="n">
-        <v>172383.175826875</v>
+        <v>267193.9225316563</v>
       </c>
       <c r="I40" s="8" t="n">
-        <v>224098.1285749375</v>
+        <v>347352.0992911531</v>
       </c>
       <c r="J40" s="8" t="n">
-        <v>246507.9414324313</v>
+        <v>382087.3092202686</v>
       </c>
       <c r="K40" s="8" t="n">
-        <v>320460.3238621607</v>
+        <v>496713.5019863491</v>
       </c>
       <c r="L40" s="8" t="n">
-        <v>416598.4210208089</v>
+        <v>645727.5525822538</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>305047</v>
+        <v>472822.85</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
@@ -2359,39 +2358,39 @@
         </is>
       </c>
       <c r="C41" s="8" t="n">
-        <v>27278.98</v>
+        <v>42282.419</v>
       </c>
       <c r="D41" s="8" t="n">
-        <v>31370.827</v>
+        <v>48624.78185000001</v>
       </c>
       <c r="E41" s="8" t="n">
-        <v>36076.45105</v>
+        <v>55918.49912750001</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>45095.5638125</v>
+        <v>69898.12390937499</v>
       </c>
       <c r="G41" s="8" t="n">
-        <v>58624.23295624999</v>
+        <v>90867.56108218749</v>
       </c>
       <c r="H41" s="8" t="n">
-        <v>76211.50284312498</v>
+        <v>118127.8294068437</v>
       </c>
       <c r="I41" s="8" t="n">
-        <v>99074.95369606248</v>
+        <v>153566.1782288968</v>
       </c>
       <c r="J41" s="8" t="n">
-        <v>108982.4490656687</v>
+        <v>168922.7960517865</v>
       </c>
       <c r="K41" s="8" t="n">
-        <v>141677.1837853693</v>
+        <v>219599.6348673224</v>
       </c>
       <c r="L41" s="8" t="n">
-        <v>184180.3389209801</v>
+        <v>285479.5253275192</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>305047</v>
+        <v>472822.85</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
@@ -2399,39 +2398,39 @@
         </is>
       </c>
       <c r="C42" s="8" t="n">
-        <v>90929.94</v>
+        <v>140941.407</v>
       </c>
       <c r="D42" s="8" t="n">
-        <v>104569.431</v>
+        <v>162082.61805</v>
       </c>
       <c r="E42" s="8" t="n">
-        <v>120254.84565</v>
+        <v>186395.0107575</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>150318.5570625</v>
+        <v>232993.763446875</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>195414.12418125</v>
+        <v>302891.8924809375</v>
       </c>
       <c r="H42" s="8" t="n">
-        <v>254038.361435625</v>
+        <v>393759.4602252188</v>
       </c>
       <c r="I42" s="8" t="n">
-        <v>330249.8698663125</v>
+        <v>511887.2982927844</v>
       </c>
       <c r="J42" s="8" t="n">
-        <v>363274.8568529438</v>
+        <v>563076.0281220629</v>
       </c>
       <c r="K42" s="8" t="n">
-        <v>472257.3139088269</v>
+        <v>731998.8365586817</v>
       </c>
       <c r="L42" s="8" t="n">
-        <v>613934.508081475</v>
+        <v>951598.4875262864</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>305101</v>
+        <v>472906.55</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
@@ -2439,39 +2438,39 @@
         </is>
       </c>
       <c r="C43" s="8" t="n">
-        <v>45524.85</v>
+        <v>70563.5175</v>
       </c>
       <c r="D43" s="8" t="n">
-        <v>52353.57749999999</v>
+        <v>81148.04512499999</v>
       </c>
       <c r="E43" s="8" t="n">
-        <v>60206.61412499999</v>
+        <v>93320.25189374998</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>75258.26765624998</v>
+        <v>116650.3148671875</v>
       </c>
       <c r="G43" s="8" t="n">
-        <v>97835.74795312498</v>
+        <v>151645.4093273437</v>
       </c>
       <c r="H43" s="8" t="n">
-        <v>127186.4723390625</v>
+        <v>197139.0321255469</v>
       </c>
       <c r="I43" s="8" t="n">
-        <v>165342.4140407813</v>
+        <v>256280.741763211</v>
       </c>
       <c r="J43" s="8" t="n">
-        <v>181876.6554448594</v>
+        <v>281908.8159395321</v>
       </c>
       <c r="K43" s="8" t="n">
-        <v>236439.6520783172</v>
+        <v>366481.4607213917</v>
       </c>
       <c r="L43" s="8" t="n">
-        <v>307371.5477018123</v>
+        <v>476425.898937809</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>305102</v>
+        <v>472908.1</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
@@ -2479,39 +2478,39 @@
         </is>
       </c>
       <c r="C44" s="8" t="n">
-        <v>29227.48</v>
+        <v>45302.594</v>
       </c>
       <c r="D44" s="8" t="n">
-        <v>33611.602</v>
+        <v>52097.9831</v>
       </c>
       <c r="E44" s="8" t="n">
-        <v>38653.3423</v>
+        <v>59912.680565</v>
       </c>
       <c r="F44" s="8" t="n">
-        <v>48316.67787499999</v>
+        <v>74890.85070624998</v>
       </c>
       <c r="G44" s="8" t="n">
-        <v>62811.68123749999</v>
+        <v>97358.10591812499</v>
       </c>
       <c r="H44" s="8" t="n">
-        <v>81655.18560874999</v>
+        <v>126565.5376935625</v>
       </c>
       <c r="I44" s="8" t="n">
-        <v>106151.741291375</v>
+        <v>164535.1990016313</v>
       </c>
       <c r="J44" s="8" t="n">
-        <v>116766.9154205125</v>
+        <v>180988.7189017944</v>
       </c>
       <c r="K44" s="8" t="n">
-        <v>151796.9900466662</v>
+        <v>235285.3345723326</v>
       </c>
       <c r="L44" s="8" t="n">
-        <v>197336.0870606661</v>
+        <v>305870.9349440325</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>425315</v>
+        <v>659238.25</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
@@ -2519,39 +2518,39 @@
         </is>
       </c>
       <c r="C45" s="8" t="n">
-        <v>29227.48</v>
+        <v>45302.594</v>
       </c>
       <c r="D45" s="8" t="n">
-        <v>33611.602</v>
+        <v>52097.9831</v>
       </c>
       <c r="E45" s="8" t="n">
-        <v>38653.3423</v>
+        <v>59912.680565</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>48316.67787499999</v>
+        <v>74890.85070624998</v>
       </c>
       <c r="G45" s="8" t="n">
-        <v>62811.68123749999</v>
+        <v>97358.10591812499</v>
       </c>
       <c r="H45" s="8" t="n">
-        <v>81655.18560874999</v>
+        <v>126565.5376935625</v>
       </c>
       <c r="I45" s="8" t="n">
-        <v>106151.741291375</v>
+        <v>164535.1990016313</v>
       </c>
       <c r="J45" s="8" t="n">
-        <v>116766.9154205125</v>
+        <v>180988.7189017944</v>
       </c>
       <c r="K45" s="8" t="n">
-        <v>151796.9900466662</v>
+        <v>235285.3345723326</v>
       </c>
       <c r="L45" s="8" t="n">
-        <v>197336.0870606661</v>
+        <v>305870.9349440325</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>500113</v>
+        <v>775175.15</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
@@ -2559,34 +2558,34 @@
         </is>
       </c>
       <c r="C46" s="8" t="n">
-        <v>20103.79</v>
+        <v>31160.8745</v>
       </c>
       <c r="D46" s="8" t="n">
-        <v>23119.3585</v>
+        <v>35835.005675</v>
       </c>
       <c r="E46" s="8" t="n">
-        <v>26587.262275</v>
+        <v>41210.25652625</v>
       </c>
       <c r="F46" s="8" t="n">
-        <v>33234.07784375</v>
+        <v>51512.8206578125</v>
       </c>
       <c r="G46" s="8" t="n">
-        <v>43204.301196875</v>
+        <v>66966.66685515625</v>
       </c>
       <c r="H46" s="8" t="n">
-        <v>56165.5915559375</v>
+        <v>87056.66691170313</v>
       </c>
       <c r="I46" s="8" t="n">
-        <v>73015.26902271876</v>
+        <v>113173.6669852141</v>
       </c>
       <c r="J46" s="8" t="n">
-        <v>80316.79592499064</v>
+        <v>124491.0336837355</v>
       </c>
       <c r="K46" s="8" t="n">
-        <v>104411.8347024878</v>
+        <v>161838.3437888561</v>
       </c>
       <c r="L46" s="8" t="n">
-        <v>135735.3851132341</v>
+        <v>210389.8469255129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
aplicar incrementos celdas combinadas
</commit_message>
<xml_diff>
--- a/PRUEBA.xlsx
+++ b/PRUEBA.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="8.28515625" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
@@ -460,6 +460,9 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -485,6 +488,15 @@
       <c r="F1" s="9" t="n">
         <v>46113</v>
       </c>
+      <c r="G1" s="9" t="n">
+        <v>46143</v>
+      </c>
+      <c r="H1" s="9" t="n">
+        <v>46174</v>
+      </c>
+      <c r="I1" s="9" t="n">
+        <v>46204</v>
+      </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -515,6 +527,21 @@
           <t xml:space="preserve"> FUERA DE CONVENIO </t>
         </is>
       </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="n">
@@ -545,6 +572,21 @@
           <t xml:space="preserve"> FUERA DE CONVENIO </t>
         </is>
       </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="n">
@@ -575,6 +617,21 @@
           <t xml:space="preserve"> FUERA DE CONVENIO </t>
         </is>
       </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -605,6 +662,21 @@
           <t xml:space="preserve"> FUERA DE CONVENIO </t>
         </is>
       </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -635,6 +707,21 @@
           <t xml:space="preserve"> FUERA DE CONVENIO </t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -657,6 +744,15 @@
       <c r="F7" s="8" t="n">
         <v>1323855.084896352</v>
       </c>
+      <c r="G7" s="8" t="n">
+        <v>1522433.347630805</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>1568106.348059729</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>1803322.300268688</v>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -687,6 +783,21 @@
           <t xml:space="preserve"> FUERA DE CONVENIO </t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -709,6 +820,15 @@
       <c r="F9" s="8" t="n">
         <v>2328234.7366764</v>
       </c>
+      <c r="G9" s="8" t="n">
+        <v>2677469.94717786</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>2757794.045593196</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>3171463.152432175</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -731,6 +851,15 @@
       <c r="F10" s="8" t="n">
         <v>1323855.084896352</v>
       </c>
+      <c r="G10" s="8" t="n">
+        <v>1522433.347630805</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>1568106.348059729</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>1803322.300268688</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -753,6 +882,15 @@
       <c r="F11" s="8" t="n">
         <v>4281576.62977152</v>
       </c>
+      <c r="G11" s="8" t="n">
+        <v>4923813.124237248</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>5071527.517964365</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>5832256.645659019</v>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2" t="n">
@@ -783,6 +921,21 @@
           <t xml:space="preserve"> FUERA DE CONVENIO </t>
         </is>
       </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="2" t="n">
@@ -813,6 +966,21 @@
           <t xml:space="preserve"> FUERA DE CONVENIO </t>
         </is>
       </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="2" t="n">
@@ -843,6 +1011,21 @@
           <t xml:space="preserve"> FUERA DE CONVENIO </t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -865,6 +1048,15 @@
       <c r="F15" s="8" t="n">
         <v>8508503.176689168</v>
       </c>
+      <c r="G15" s="8" t="n">
+        <v>9784778.653192542</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>10078322.01278832</v>
+      </c>
+      <c r="I15" s="8" t="n">
+        <v>11590070.31470657</v>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="2" t="n">
@@ -895,6 +1087,21 @@
           <t xml:space="preserve"> FUERA DE CONVENIO </t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -917,6 +1124,15 @@
       <c r="F17" s="8" t="n">
         <v>14560998.07280803</v>
       </c>
+      <c r="G17" s="8" t="n">
+        <v>16745147.78372923</v>
+      </c>
+      <c r="H17" s="8" t="n">
+        <v>17247502.2172411</v>
+      </c>
+      <c r="I17" s="8" t="n">
+        <v>19834627.54982726</v>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2" t="n">
@@ -947,6 +1163,21 @@
           <t xml:space="preserve"> FUERA DE CONVENIO </t>
         </is>
       </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -969,6 +1200,15 @@
       <c r="F19" s="8" t="n">
         <v>7293002.687498592</v>
       </c>
+      <c r="G19" s="8" t="n">
+        <v>8386953.09062338</v>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>8638561.683342081</v>
+      </c>
+      <c r="I19" s="8" t="n">
+        <v>9934345.935843391</v>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="2" t="n">
@@ -999,6 +1239,21 @@
           <t xml:space="preserve"> FUERA DE CONVENIO </t>
         </is>
       </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="2" t="n">
@@ -1029,6 +1284,21 @@
           <t xml:space="preserve"> FUERA DE CONVENIO </t>
         </is>
       </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1051,6 +1321,15 @@
       <c r="F22" s="8" t="n">
         <v>1810400.163192432</v>
       </c>
+      <c r="G22" s="8" t="n">
+        <v>2081960.187671297</v>
+      </c>
+      <c r="H22" s="8" t="n">
+        <v>2144418.993301436</v>
+      </c>
+      <c r="I22" s="8" t="n">
+        <v>2466081.842296651</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1073,6 +1352,15 @@
       <c r="F23" s="8" t="n">
         <v>1584100.119576672</v>
       </c>
+      <c r="G23" s="8" t="n">
+        <v>1821715.137513173</v>
+      </c>
+      <c r="H23" s="8" t="n">
+        <v>1876366.591638568</v>
+      </c>
+      <c r="I23" s="8" t="n">
+        <v>2157821.580384353</v>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="2" t="n">
@@ -1103,6 +1391,21 @@
           <t xml:space="preserve"> FUERA DE CONVENIO </t>
         </is>
       </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> FUERA DE CONVENIO </t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1125,6 +1428,15 @@
       <c r="F25" s="8" t="n">
         <v>17572341.66479539</v>
       </c>
+      <c r="G25" s="8" t="n">
+        <v>20208192.9145147</v>
+      </c>
+      <c r="H25" s="8" t="n">
+        <v>20814438.70195014</v>
+      </c>
+      <c r="I25" s="8" t="n">
+        <v>23936604.50724266</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1147,6 +1459,15 @@
       <c r="F26" s="8" t="n">
         <v>261373.490414352</v>
       </c>
+      <c r="G26" s="8" t="n">
+        <v>300579.5139765048</v>
+      </c>
+      <c r="H26" s="8" t="n">
+        <v>309596.8993958</v>
+      </c>
+      <c r="I26" s="8" t="n">
+        <v>356036.43430517</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1169,6 +1490,15 @@
       <c r="F27" s="8" t="n">
         <v>261373.490414352</v>
       </c>
+      <c r="G27" s="8" t="n">
+        <v>300579.5139765048</v>
+      </c>
+      <c r="H27" s="8" t="n">
+        <v>309596.8993958</v>
+      </c>
+      <c r="I27" s="8" t="n">
+        <v>356036.43430517</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1191,6 +1521,15 @@
       <c r="F28" s="8" t="n">
         <v>141437.534998752</v>
       </c>
+      <c r="G28" s="8" t="n">
+        <v>162653.1652485648</v>
+      </c>
+      <c r="H28" s="8" t="n">
+        <v>167532.7602060217</v>
+      </c>
+      <c r="I28" s="8" t="n">
+        <v>192662.6742369249</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1213,6 +1552,15 @@
       <c r="F29" s="8" t="n">
         <v>261373.490414352</v>
       </c>
+      <c r="G29" s="8" t="n">
+        <v>300579.5139765048</v>
+      </c>
+      <c r="H29" s="8" t="n">
+        <v>309596.8993958</v>
+      </c>
+      <c r="I29" s="8" t="n">
+        <v>356036.43430517</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1235,6 +1583,15 @@
       <c r="F30" s="8" t="n">
         <v>180950.882741568</v>
       </c>
+      <c r="G30" s="8" t="n">
+        <v>208093.5151528032</v>
+      </c>
+      <c r="H30" s="8" t="n">
+        <v>214336.3206073873</v>
+      </c>
+      <c r="I30" s="8" t="n">
+        <v>246486.7686984953</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1257,6 +1614,15 @@
       <c r="F31" s="8" t="n">
         <v>180950.882741568</v>
       </c>
+      <c r="G31" s="8" t="n">
+        <v>208093.5151528032</v>
+      </c>
+      <c r="H31" s="8" t="n">
+        <v>214336.3206073873</v>
+      </c>
+      <c r="I31" s="8" t="n">
+        <v>246486.7686984953</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -1279,6 +1645,15 @@
       <c r="F32" s="8" t="n">
         <v>180950.882741568</v>
       </c>
+      <c r="G32" s="8" t="n">
+        <v>208093.5151528032</v>
+      </c>
+      <c r="H32" s="8" t="n">
+        <v>214336.3206073873</v>
+      </c>
+      <c r="I32" s="8" t="n">
+        <v>246486.7686984953</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -1301,6 +1676,15 @@
       <c r="F33" s="8" t="n">
         <v>180950.882741568</v>
       </c>
+      <c r="G33" s="8" t="n">
+        <v>208093.5151528032</v>
+      </c>
+      <c r="H33" s="8" t="n">
+        <v>214336.3206073873</v>
+      </c>
+      <c r="I33" s="8" t="n">
+        <v>246486.7686984953</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -1323,6 +1707,15 @@
       <c r="F34" s="8" t="n">
         <v>402113.100275136</v>
       </c>
+      <c r="G34" s="8" t="n">
+        <v>462430.0653164064</v>
+      </c>
+      <c r="H34" s="8" t="n">
+        <v>476302.9672758986</v>
+      </c>
+      <c r="I34" s="8" t="n">
+        <v>547748.4123672834</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -1345,6 +1738,15 @@
       <c r="F35" s="8" t="n">
         <v>603169.650412704</v>
       </c>
+      <c r="G35" s="8" t="n">
+        <v>693645.0979746095</v>
+      </c>
+      <c r="H35" s="8" t="n">
+        <v>714454.4509138478</v>
+      </c>
+      <c r="I35" s="8" t="n">
+        <v>821622.6185509249</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -1367,6 +1769,15 @@
       <c r="F36" s="8" t="n">
         <v>261373.490414352</v>
       </c>
+      <c r="G36" s="8" t="n">
+        <v>300579.5139765048</v>
+      </c>
+      <c r="H36" s="8" t="n">
+        <v>309596.8993958</v>
+      </c>
+      <c r="I36" s="8" t="n">
+        <v>356036.43430517</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -1389,6 +1800,15 @@
       <c r="F37" s="8" t="n">
         <v>442324.3731559199</v>
       </c>
+      <c r="G37" s="8" t="n">
+        <v>508673.0291293078</v>
+      </c>
+      <c r="H37" s="8" t="n">
+        <v>523933.220003187</v>
+      </c>
+      <c r="I37" s="8" t="n">
+        <v>602523.203003665</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -1411,6 +1831,15 @@
       <c r="F38" s="8" t="n">
         <v>502641.37534392</v>
       </c>
+      <c r="G38" s="8" t="n">
+        <v>578037.5816455079</v>
+      </c>
+      <c r="H38" s="8" t="n">
+        <v>595378.7090948732</v>
+      </c>
+      <c r="I38" s="8" t="n">
+        <v>684685.5154591041</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -1433,6 +1862,15 @@
       <c r="F39" s="8" t="n">
         <v>251320.780538784</v>
       </c>
+      <c r="G39" s="8" t="n">
+        <v>289018.8976196016</v>
+      </c>
+      <c r="H39" s="8" t="n">
+        <v>297689.4645481896</v>
+      </c>
+      <c r="I39" s="8" t="n">
+        <v>342342.884230418</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -1455,6 +1893,15 @@
       <c r="F40" s="8" t="n">
         <v>382007.432879136</v>
       </c>
+      <c r="G40" s="8" t="n">
+        <v>439308.5478110064</v>
+      </c>
+      <c r="H40" s="8" t="n">
+        <v>452487.8042453366</v>
+      </c>
+      <c r="I40" s="8" t="n">
+        <v>520360.9748821371</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -1477,6 +1924,15 @@
       <c r="F41" s="8" t="n">
         <v>168887.482303968</v>
       </c>
+      <c r="G41" s="8" t="n">
+        <v>194220.6046495632</v>
+      </c>
+      <c r="H41" s="8" t="n">
+        <v>200047.2227890501</v>
+      </c>
+      <c r="I41" s="8" t="n">
+        <v>230054.3062074076</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -1499,6 +1955,15 @@
       <c r="F42" s="8" t="n">
         <v>562958.3156207041</v>
       </c>
+      <c r="G42" s="8" t="n">
+        <v>647402.0629638097</v>
+      </c>
+      <c r="H42" s="8" t="n">
+        <v>666824.124852724</v>
+      </c>
+      <c r="I42" s="8" t="n">
+        <v>766847.7435806326</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -1521,6 +1986,15 @@
       <c r="F43" s="8" t="n">
         <v>281849.88217176</v>
       </c>
+      <c r="G43" s="8" t="n">
+        <v>324127.364497524</v>
+      </c>
+      <c r="H43" s="8" t="n">
+        <v>333851.1854324497</v>
+      </c>
+      <c r="I43" s="8" t="n">
+        <v>383928.8632473171</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -1543,6 +2017,15 @@
       <c r="F44" s="8" t="n">
         <v>180950.882741568</v>
       </c>
+      <c r="G44" s="8" t="n">
+        <v>208093.5151528032</v>
+      </c>
+      <c r="H44" s="8" t="n">
+        <v>214336.3206073873</v>
+      </c>
+      <c r="I44" s="8" t="n">
+        <v>246486.7686984953</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -1565,6 +2048,15 @@
       <c r="F45" s="8" t="n">
         <v>180950.882741568</v>
       </c>
+      <c r="G45" s="8" t="n">
+        <v>208093.5151528032</v>
+      </c>
+      <c r="H45" s="8" t="n">
+        <v>214336.3206073873</v>
+      </c>
+      <c r="I45" s="8" t="n">
+        <v>246486.7686984953</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -1586,6 +2078,15 @@
       </c>
       <c r="F46" s="8" t="n">
         <v>124465.008510864</v>
+      </c>
+      <c r="G46" s="8" t="n">
+        <v>143134.7597874936</v>
+      </c>
+      <c r="H46" s="8" t="n">
+        <v>147428.8025811184</v>
+      </c>
+      <c r="I46" s="8" t="n">
+        <v>169543.1229682861</v>
       </c>
     </row>
   </sheetData>

</xml_diff>